<commit_message>
Upated FigureDrawer to handle our new ExternalGCp curve format
-- updated drawing functions
-- minor UI visual improvements
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/VerificationSpreadsheet.xlsx
+++ b/WindLoadCalculations/VerificationSpreadsheet.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7004A53A-686B-40D1-B67F-25EB4762B319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B33496-9F31-4AB5-B4E6-3461C9254E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="885" yWindow="480" windowWidth="26460" windowHeight="14130" activeTab="1" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
+    <workbookView xWindow="-27060" yWindow="810" windowWidth="26460" windowHeight="14130" activeTab="1" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
   </bookViews>
   <sheets>
     <sheet name="Exposure C" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2758,4 +2759,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD8320E2-F01C-4F60-9B3D-82EC74076ADF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed defaults in WindLoadInputControl
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/VerificationSpreadsheet.xlsx
+++ b/WindLoadCalculations/VerificationSpreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B33496-9F31-4AB5-B4E6-3461C9254E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD34F51-3A1E-4FA5-93C5-538BA445BC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27060" yWindow="810" windowWidth="26460" windowHeight="14130" activeTab="1" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
+    <workbookView xWindow="-28245" yWindow="660" windowWidth="26460" windowHeight="14130" activeTab="1" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
   </bookViews>
   <sheets>
     <sheet name="Exposure C" sheetId="1" r:id="rId1"/>
@@ -2535,18 +2535,18 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>0.26100000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="F14">
-        <v>-2.5</v>
+        <v>-2.5499999999999998</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>10.861776000000001</v>
+        <v>9.5716800000000006</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>-104.03999999999999</v>
+        <v>-106.12079999999999</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
@@ -2558,11 +2558,11 @@
       </c>
       <c r="L14">
         <f t="shared" si="4"/>
-        <v>18.352656</v>
+        <v>17.062560000000001</v>
       </c>
       <c r="M14">
         <f t="shared" si="5"/>
-        <v>-111.53088</v>
+        <v>-113.61167999999999</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15">

</xml_diff>

<commit_message>
Fixed an error in the mean roof height calculation for hips and gables
-- mean roof height is half the height of the sloped region, not the topmost point
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/VerificationSpreadsheet.xlsx
+++ b/WindLoadCalculations/VerificationSpreadsheet.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E668DF37-2661-40C7-A2D7-57252180E9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78B4F1C-D5B9-4837-9C78-02618DB4DFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23985" yWindow="285" windowWidth="22905" windowHeight="14130" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
+    <workbookView xWindow="-25455" yWindow="645" windowWidth="22905" windowHeight="14130" activeTab="3" xr2:uid="{7D93B743-C6BA-493F-B145-C673A908EA6D}"/>
   </bookViews>
   <sheets>
     <sheet name="ASCE7-16 ExpC" sheetId="1" r:id="rId1"/>
     <sheet name="ASCE7-22 ExpC" sheetId="5" r:id="rId2"/>
     <sheet name="40x60 FLAT ASCE7-16" sheetId="2" r:id="rId3"/>
     <sheet name="40x60 GABLE ASCE7-16" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId5"/>
+    <sheet name="40x60 HIP ASCE7-16" sheetId="6" r:id="rId5"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="148">
   <si>
     <t>TDI Data Values</t>
   </si>
@@ -391,13 +392,106 @@
   </si>
   <si>
     <t>&lt;--- EXCEEDS 60 ft forChapter30 Figures</t>
+  </si>
+  <si>
+    <t>2e_B</t>
+  </si>
+  <si>
+    <t>2e_L</t>
+  </si>
+  <si>
+    <t>(B-2a)*a</t>
+  </si>
+  <si>
+    <t>2r_L</t>
+  </si>
+  <si>
+    <t>2r_B</t>
+  </si>
+  <si>
+    <t>1_L</t>
+  </si>
+  <si>
+    <t>0.5*(2L-B)*0.5*B</t>
+  </si>
+  <si>
+    <t>b =</t>
+  </si>
+  <si>
+    <t>1.414*a</t>
+  </si>
+  <si>
+    <t>c =</t>
+  </si>
+  <si>
+    <t>B/2-2a</t>
+  </si>
+  <si>
+    <t>Area L-side Trapezoid</t>
+  </si>
+  <si>
+    <t>0.5*(2L-4b-4a-2c)*c</t>
+  </si>
+  <si>
+    <t>A_trap-A3-A2e-A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d = </t>
+  </si>
+  <si>
+    <t>Longside (trapezoid)</t>
+  </si>
+  <si>
+    <t>ShortSide(triangle)</t>
+  </si>
+  <si>
+    <t>B (short side)</t>
+  </si>
+  <si>
+    <t>L (long side)</t>
+  </si>
+  <si>
+    <t>1_B</t>
+  </si>
+  <si>
+    <t>B/2-b-a</t>
+  </si>
+  <si>
+    <t>Area B-side Triangle</t>
+  </si>
+  <si>
+    <t>0.5*B*0.5*B</t>
+  </si>
+  <si>
+    <t>0.5*(B-2a-2b)*d</t>
+  </si>
+  <si>
+    <t>A_tri-A3-A2e-A1</t>
+  </si>
+  <si>
+    <t>SUBTOTAL (2 similar) =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">h/B = </t>
+  </si>
+  <si>
+    <t>HIP VERIFICATION - ASCE7-16</t>
+  </si>
+  <si>
+    <t>17.5'</t>
+  </si>
+  <si>
+    <t>z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -420,6 +514,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="1"/>
@@ -427,7 +527,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -446,8 +546,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -481,11 +587,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -497,7 +612,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2098,6 +2223,9 @@
       <c r="E23" t="s">
         <v>24</v>
       </c>
+      <c r="G23">
+        <v>20.36</v>
+      </c>
     </row>
     <row r="24" spans="1:33">
       <c r="A24">
@@ -7207,6 +7335,12 @@
       <c r="L3" s="5">
         <v>0.85</v>
       </c>
+      <c r="N3" t="s">
+        <v>77</v>
+      </c>
+      <c r="O3" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="4" spans="1:15" ht="15">
       <c r="A4" s="1" t="s">
@@ -7223,14 +7357,14 @@
       </c>
       <c r="F4">
         <f>MIN(H4,H5)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G4" t="s">
         <v>57</v>
       </c>
       <c r="H4">
         <f>0.4*B7</f>
-        <v>8.1424555792624798</v>
+        <v>0</v>
       </c>
       <c r="I4" t="s">
         <v>1</v>
@@ -7239,7 +7373,7 @@
         <v>77</v>
       </c>
       <c r="L4" s="5">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="N4">
         <v>0.85</v>
@@ -7269,10 +7403,10 @@
         <v>1</v>
       </c>
       <c r="N5">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="O5" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="15" thickBot="1">
@@ -7307,16 +7441,16 @@
       </c>
       <c r="L6" s="4">
         <f>0.00256*B9*B9*L4*L3</f>
-        <v>44.553600000000003</v>
+        <v>43.084800000000001</v>
       </c>
       <c r="M6" t="s">
         <v>41</v>
       </c>
       <c r="N6">
-        <v>0.96</v>
+        <v>0.91</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="15" thickBot="1">
@@ -7324,8 +7458,8 @@
         <v>58</v>
       </c>
       <c r="B7" s="7">
-        <f>$B$6+TAN($B$8 * 6.28 / 360)*$B$4/2</f>
-        <v>20.356138948156197</v>
+        <f>D7</f>
+        <v>0</v>
       </c>
       <c r="C7" t="s">
         <v>1</v>
@@ -7338,6 +7472,12 @@
       </c>
       <c r="I7" t="s">
         <v>1</v>
+      </c>
+      <c r="N7">
+        <v>0.96</v>
+      </c>
+      <c r="O7" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="15" thickBot="1">
@@ -7355,7 +7495,7 @@
       </c>
       <c r="F8" s="4">
         <f>MAX(F6,F4)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="s">
         <v>1</v>
@@ -7439,7 +7579,7 @@
       </c>
       <c r="C13">
         <f>F8*F8</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E13">
         <v>0.48</v>
@@ -7449,27 +7589,27 @@
       </c>
       <c r="G13">
         <f>$L$6*E13</f>
-        <v>21.385728</v>
+        <v>20.680703999999999</v>
       </c>
       <c r="H13">
         <f>$L$6*F13</f>
-        <v>-122.07686400000001</v>
+        <v>-118.05235200000001</v>
       </c>
       <c r="I13">
         <f>$L$6*$L$2</f>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J13">
         <f>-$L$6*$L$2</f>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L13">
         <f>G13+I13</f>
-        <v>29.405376</v>
+        <v>28.435967999999999</v>
       </c>
       <c r="M13">
         <f>H13+J13</f>
-        <v>-130.09651200000002</v>
+        <v>-125.80761600000001</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -7481,7 +7621,7 @@
       </c>
       <c r="C14">
         <f>F8*F8</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E14">
         <v>0.5</v>
@@ -7491,27 +7631,27 @@
       </c>
       <c r="G14">
         <f t="shared" ref="G14:G18" si="0">$L$6*E14</f>
-        <v>22.276800000000001</v>
+        <v>21.542400000000001</v>
       </c>
       <c r="H14">
         <f t="shared" ref="H14:H18" si="1">$L$6*F14</f>
-        <v>-149.25456000000003</v>
+        <v>-144.33408</v>
       </c>
       <c r="I14">
         <f t="shared" ref="I14:I18" si="2">$L$6*$L$2</f>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J14">
         <f t="shared" ref="J14:J18" si="3">-$L$6*$L$2</f>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L14">
         <f t="shared" ref="L14:L18" si="4">G14+I14</f>
-        <v>30.296448000000002</v>
+        <v>29.297664000000001</v>
       </c>
       <c r="M14">
         <f t="shared" ref="M14:M18" si="5">H14+J14</f>
-        <v>-157.27420800000002</v>
+        <v>-152.08934400000001</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -7523,7 +7663,7 @@
       </c>
       <c r="C15">
         <f>(B4/2-2*F8)*F8</f>
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E15">
         <v>0.38</v>
@@ -7533,27 +7673,27 @@
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>16.930368000000001</v>
+        <v>16.372223999999999</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
-        <v>-89.998272</v>
+        <v>-87.031295999999998</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J15">
         <f t="shared" si="3"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L15">
         <f t="shared" si="4"/>
-        <v>24.950016000000002</v>
+        <v>24.127488</v>
       </c>
       <c r="M15">
         <f t="shared" si="5"/>
-        <v>-98.017920000000004</v>
+        <v>-94.786559999999994</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -7565,7 +7705,7 @@
       </c>
       <c r="C16">
         <f>(B5-2*F8)*F8</f>
-        <v>208</v>
+        <v>162</v>
       </c>
       <c r="E16">
         <v>0.3</v>
@@ -7575,27 +7715,27 @@
       </c>
       <c r="G16">
         <f t="shared" si="0"/>
-        <v>13.36608</v>
+        <v>12.92544</v>
       </c>
       <c r="H16">
         <f t="shared" si="1"/>
-        <v>-22.276800000000001</v>
+        <v>-21.542400000000001</v>
       </c>
       <c r="I16">
         <f t="shared" si="2"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J16">
         <f t="shared" si="3"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L16">
         <f t="shared" si="4"/>
-        <v>21.385728</v>
+        <v>20.680703999999999</v>
       </c>
       <c r="M16">
         <f t="shared" si="5"/>
-        <v>-30.296448000000002</v>
+        <v>-29.297664000000001</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7607,7 +7747,7 @@
       </c>
       <c r="C17">
         <f>(B5-2*$F$8)*$F$8</f>
-        <v>208</v>
+        <v>162</v>
       </c>
       <c r="E17">
         <v>0.3</v>
@@ -7617,27 +7757,27 @@
       </c>
       <c r="G17">
         <f t="shared" si="0"/>
-        <v>13.36608</v>
+        <v>12.92544</v>
       </c>
       <c r="H17">
         <f t="shared" si="1"/>
-        <v>-49.008960000000009</v>
+        <v>-47.393280000000004</v>
       </c>
       <c r="I17">
         <f t="shared" si="2"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J17">
         <f t="shared" si="3"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L17">
         <f t="shared" si="4"/>
-        <v>21.385728</v>
+        <v>20.680703999999999</v>
       </c>
       <c r="M17">
         <f t="shared" si="5"/>
-        <v>-57.028608000000006</v>
+        <v>-55.148544000000001</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -7649,7 +7789,7 @@
       </c>
       <c r="C18">
         <f>($B$5*$B$4/2)-2*C13-2*C14-2*C15-C16-C17</f>
-        <v>624</v>
+        <v>756</v>
       </c>
       <c r="E18">
         <v>0.3</v>
@@ -7659,27 +7799,27 @@
       </c>
       <c r="G18">
         <f t="shared" si="0"/>
-        <v>13.36608</v>
+        <v>12.92544</v>
       </c>
       <c r="H18">
         <f t="shared" si="1"/>
-        <v>-22.276800000000001</v>
+        <v>-21.542400000000001</v>
       </c>
       <c r="I18">
         <f t="shared" si="2"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J18">
         <f t="shared" si="3"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L18">
         <f t="shared" si="4"/>
-        <v>21.385728</v>
+        <v>20.680703999999999</v>
       </c>
       <c r="M18">
         <f t="shared" si="5"/>
-        <v>-30.296448000000002</v>
+        <v>-29.297664000000001</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="15">
@@ -7709,7 +7849,7 @@
       </c>
       <c r="C22">
         <f>F8*B6</f>
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E22">
         <v>0.83</v>
@@ -7719,27 +7859,27 @@
       </c>
       <c r="G22">
         <f>$L$6*E22</f>
-        <v>36.979488000000003</v>
+        <v>35.760384000000002</v>
       </c>
       <c r="H22">
         <f>$L$6*F22</f>
-        <v>-50.345568</v>
+        <v>-48.685823999999997</v>
       </c>
       <c r="I22">
         <f t="shared" ref="I22:I24" si="6">$L$6*$L$2</f>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J22">
         <f t="shared" ref="J22:J24" si="7">-$L$6*$L$2</f>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L22">
         <f>G22+I22</f>
-        <v>44.999136000000007</v>
+        <v>43.515647999999999</v>
       </c>
       <c r="M22">
         <f>H22+J22</f>
-        <v>-58.365216000000004</v>
+        <v>-56.441087999999993</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -7751,7 +7891,7 @@
       </c>
       <c r="C23">
         <f>($B$5-2*$F$8)*($B$6)</f>
-        <v>780</v>
+        <v>810</v>
       </c>
       <c r="E23">
         <v>0.71</v>
@@ -7761,27 +7901,27 @@
       </c>
       <c r="G23">
         <f>$L$6*E23</f>
-        <v>31.633056</v>
+        <v>30.590208000000001</v>
       </c>
       <c r="H23">
         <f>$L$6*F23</f>
-        <v>-35.642880000000005</v>
+        <v>-34.467840000000002</v>
       </c>
       <c r="I23">
         <f t="shared" si="6"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J23">
         <f t="shared" si="7"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L23">
         <f>G23+I23</f>
-        <v>39.652704</v>
+        <v>38.345472000000001</v>
       </c>
       <c r="M23">
         <f>H23+J23</f>
-        <v>-43.662528000000009</v>
+        <v>-42.223104000000006</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="15">
@@ -7798,7 +7938,7 @@
       </c>
       <c r="C26">
         <f>0.5*($B$6+$B$6+$F$8*TAN(RADIANS($B$8)))*$F$8</f>
-        <v>62.143593539448979</v>
+        <v>46.205771365940052</v>
       </c>
       <c r="E26">
         <v>0.83</v>
@@ -7808,27 +7948,27 @@
       </c>
       <c r="G26">
         <f>$L$6*E26</f>
-        <v>36.979488000000003</v>
+        <v>35.760384000000002</v>
       </c>
       <c r="H26">
         <f>$L$6*F26</f>
-        <v>-50.345568</v>
+        <v>-48.685823999999997</v>
       </c>
       <c r="I26">
         <f t="shared" ref="I26:I28" si="8">$L$6*$L$2</f>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J26">
         <f t="shared" ref="J26:J28" si="9">-$L$6*$L$2</f>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L26">
         <f>G26+I26</f>
-        <v>44.999136000000007</v>
+        <v>43.515647999999999</v>
       </c>
       <c r="M26">
         <f>H26+J26</f>
-        <v>-58.365216000000004</v>
+        <v>-56.441087999999993</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -7837,7 +7977,7 @@
       </c>
       <c r="C27">
         <f>($B$6*$B$4)+0.5*$B$4/2*TAN(RADIANS(B8))*$B$4  - 2*C26</f>
-        <v>582.8924898935511</v>
+        <v>614.768134240569</v>
       </c>
       <c r="E27">
         <v>0.7</v>
@@ -7847,27 +7987,27 @@
       </c>
       <c r="G27">
         <f>$L$6*E27</f>
-        <v>31.187519999999999</v>
+        <v>30.15936</v>
       </c>
       <c r="H27">
         <f>$L$6*F27</f>
-        <v>-35.642880000000005</v>
+        <v>-34.467840000000002</v>
       </c>
       <c r="I27">
         <f t="shared" si="8"/>
-        <v>8.0196480000000001</v>
+        <v>7.7552640000000004</v>
       </c>
       <c r="J27">
         <f t="shared" si="9"/>
-        <v>-8.0196480000000001</v>
+        <v>-7.7552640000000004</v>
       </c>
       <c r="L27">
         <f>G27+I27</f>
-        <v>39.207167999999996</v>
+        <v>37.914624000000003</v>
       </c>
       <c r="M27">
         <f>H27+J27</f>
-        <v>-43.662528000000009</v>
+        <v>-42.223104000000006</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7877,7 +8017,7 @@
       </c>
       <c r="C30">
         <f>B30*F8</f>
-        <v>1.0712277896312392</v>
+        <v>0.80342084222342947</v>
       </c>
     </row>
   </sheetData>
@@ -7886,6 +8026,903 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A07C503-ABDA-4895-82E4-84650588D8A5}">
+  <dimension ref="A1:O45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="18.625" customWidth="1"/>
+    <col min="2" max="2" width="33.75" customWidth="1"/>
+    <col min="7" max="7" width="12.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="15">
+      <c r="A1" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" s="5">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L3" s="5">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="5">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4">
+        <f>MIN(H4,H5)</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4">
+        <f>0.4*B7</f>
+        <v>8.1424555792624798</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>77</v>
+      </c>
+      <c r="L4" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="N4">
+        <v>0.85</v>
+      </c>
+      <c r="O4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="15" thickBot="1">
+      <c r="A5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="5">
+        <v>60</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5">
+        <f>0.1*MIN(B4,B5)</f>
+        <v>4</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>0.91</v>
+      </c>
+      <c r="O5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="15" thickBot="1">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="5">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6">
+        <f>MAX(H6:H7)</f>
+        <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6">
+        <f>0.04*MIN(B4,B5)</f>
+        <v>1.6</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="4">
+        <f>0.00256*B9*B9*L4*L3</f>
+        <v>44.553600000000003</v>
+      </c>
+      <c r="M6" t="s">
+        <v>41</v>
+      </c>
+      <c r="N6">
+        <v>0.96</v>
+      </c>
+      <c r="O6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="15" thickBot="1">
+      <c r="A7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="12">
+        <f>$B$6+TAN($B$8 * 6.28 / 360)*$B$4/2</f>
+        <v>20.356138948156197</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="15" thickBot="1">
+      <c r="A8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="5">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="4">
+        <f>MAX(F6,F4)</f>
+        <v>4</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="5">
+        <v>150</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9">
+        <f>B7/B4</f>
+        <v>0.50890347370390487</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="B10" s="5"/>
+    </row>
+    <row r="11" spans="1:15" ht="15">
+      <c r="A11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G11" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" t="s">
+        <v>81</v>
+      </c>
+      <c r="I11" t="s">
+        <v>82</v>
+      </c>
+      <c r="J11" t="s">
+        <v>83</v>
+      </c>
+      <c r="L11" t="s">
+        <v>89</v>
+      </c>
+      <c r="M11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="15">
+      <c r="A12" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" t="s">
+        <v>84</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="L12" t="s">
+        <v>41</v>
+      </c>
+      <c r="M12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="16">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13">
+        <f>F8*F8</f>
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>0.65</v>
+      </c>
+      <c r="F13">
+        <v>-1.7</v>
+      </c>
+      <c r="G13">
+        <f>$L$6*E13</f>
+        <v>28.959840000000003</v>
+      </c>
+      <c r="H13">
+        <f>$L$6*F13</f>
+        <v>-75.741120000000009</v>
+      </c>
+      <c r="I13">
+        <f>$L$6*$L$2</f>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J13">
+        <f>-$L$6*$L$2</f>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L13">
+        <f>G13+I13</f>
+        <v>36.979488000000003</v>
+      </c>
+      <c r="M13">
+        <f>H13+J13</f>
+        <v>-83.760768000000013</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14">
+        <f>(B5-2*F8)*F8</f>
+        <v>208</v>
+      </c>
+      <c r="E14">
+        <v>0.3</v>
+      </c>
+      <c r="F14">
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="G14">
+        <f t="shared" ref="G14:H33" si="0">$L$6*E14</f>
+        <v>13.36608</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>-49.008960000000009</v>
+      </c>
+      <c r="I14">
+        <f t="shared" ref="I14:I33" si="1">$L$6*$L$2</f>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J14">
+        <f t="shared" ref="J14:J33" si="2">-$L$6*$L$2</f>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L14">
+        <f t="shared" ref="L14:M33" si="3">G14+I14</f>
+        <v>21.385728</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="3"/>
+        <v>-57.028608000000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15">
+        <f>C27-C13-C14-C16</f>
+        <v>231.74399999999997</v>
+      </c>
+      <c r="E15">
+        <v>0.3</v>
+      </c>
+      <c r="F15">
+        <v>-1.3</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>13.36608</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>-57.919680000000007</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="3"/>
+        <v>21.385728</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="3"/>
+        <v>-65.939328000000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" s="14">
+        <f>0.5*((B5-2*C29-2*F8)+(B5-2*F8-2*C29-2*C30))*C30</f>
+        <v>344.25600000000003</v>
+      </c>
+      <c r="E16">
+        <v>0.3</v>
+      </c>
+      <c r="F16">
+        <v>-1</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>13.36608</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="0"/>
+        <v>-44.553600000000003</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="3"/>
+        <v>21.385728</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="3"/>
+        <v>-52.573248000000007</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="B17" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17">
+        <f>2*SUM(C13:C16)</f>
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="15">
+      <c r="A19" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="16">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>101</v>
+      </c>
+      <c r="C20">
+        <f>F8*F8</f>
+        <v>16</v>
+      </c>
+      <c r="E20">
+        <v>0.65</v>
+      </c>
+      <c r="F20">
+        <v>-1.7</v>
+      </c>
+      <c r="G20">
+        <f t="shared" ref="G17:G20" si="4">$L$6*E20</f>
+        <v>28.959840000000003</v>
+      </c>
+      <c r="H20">
+        <f t="shared" ref="H17:H20" si="5">$L$6*F20</f>
+        <v>-75.741120000000009</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L20">
+        <f t="shared" ref="L17:L20" si="6">G20+I20</f>
+        <v>36.979488000000003</v>
+      </c>
+      <c r="M20">
+        <f t="shared" ref="M17:M20" si="7">H20+J20</f>
+        <v>-83.760768000000013</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21">
+        <f>(B4-2*$F$8)*$F$8</f>
+        <v>128</v>
+      </c>
+      <c r="E21">
+        <v>0.3</v>
+      </c>
+      <c r="F21">
+        <v>-1.23</v>
+      </c>
+      <c r="G21">
+        <f t="shared" ref="G21:G23" si="8">$L$6*E21</f>
+        <v>13.36608</v>
+      </c>
+      <c r="H21">
+        <f t="shared" ref="H21:H23" si="9">$L$6*F21</f>
+        <v>-54.800928000000006</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L21">
+        <f t="shared" ref="L21:L23" si="10">G21+I21</f>
+        <v>21.385728</v>
+      </c>
+      <c r="M21">
+        <f t="shared" ref="M21:M23" si="11">H21+J21</f>
+        <v>-62.820576000000003</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22">
+        <f>C28-C20-C21-C23</f>
+        <v>149.00166399999998</v>
+      </c>
+      <c r="E22">
+        <v>0.3</v>
+      </c>
+      <c r="F22">
+        <v>-1.4</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="8"/>
+        <v>13.36608</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="9"/>
+        <v>-62.375039999999998</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="10"/>
+        <v>21.385728</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="11"/>
+        <v>-70.394688000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C23" s="14">
+        <f>0.5*(B4-2*F8-2*C29)*C31</f>
+        <v>106.99833600000002</v>
+      </c>
+      <c r="E23">
+        <v>0.3</v>
+      </c>
+      <c r="F23">
+        <v>-1</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="8"/>
+        <v>13.36608</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="9"/>
+        <v>-44.553600000000003</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="1"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="2"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="10"/>
+        <v>21.385728</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="11"/>
+        <v>-52.573248000000007</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="B24" t="s">
+        <v>142</v>
+      </c>
+      <c r="C24">
+        <f>2*SUM(C20:C23)</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15">
+      <c r="B25" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C25" s="1">
+        <f>C17+C24</f>
+        <v>2400</v>
+      </c>
+      <c r="D25" s="1" t="str">
+        <f>IF(C25=B4*B5,"OK","N.G.")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C27">
+        <f>0.5*(2*B5-B4)*0.5*B4</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" t="s">
+        <v>138</v>
+      </c>
+      <c r="B28" t="s">
+        <v>139</v>
+      </c>
+      <c r="C28">
+        <f>0.5*B4*0.5*B4</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29">
+        <f>1.414*F8</f>
+        <v>5.6559999999999997</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30">
+        <f>B4/2-2*F8</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" t="s">
+        <v>131</v>
+      </c>
+      <c r="B31" t="s">
+        <v>137</v>
+      </c>
+      <c r="C31">
+        <f>0.5*B4-C29-F8</f>
+        <v>10.344000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="15">
+      <c r="C34" s="1"/>
+    </row>
+    <row r="36" spans="1:13" ht="15">
+      <c r="A36" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37">
+        <v>5</v>
+      </c>
+      <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37">
+        <f>F8*B6</f>
+        <v>60</v>
+      </c>
+      <c r="E37">
+        <v>0.83</v>
+      </c>
+      <c r="F37">
+        <v>-1.1299999999999999</v>
+      </c>
+      <c r="G37">
+        <f>$L$6*E37</f>
+        <v>36.979488000000003</v>
+      </c>
+      <c r="H37">
+        <f>$L$6*F37</f>
+        <v>-50.345568</v>
+      </c>
+      <c r="I37">
+        <f t="shared" ref="I37:I39" si="12">$L$6*$L$2</f>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J37">
+        <f t="shared" ref="J37:J39" si="13">-$L$6*$L$2</f>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L37">
+        <f>G37+I37</f>
+        <v>44.999136000000007</v>
+      </c>
+      <c r="M37">
+        <f>H37+J37</f>
+        <v>-58.365216000000004</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38">
+        <f>($B$5-2*$F$8)*($B$6)</f>
+        <v>780</v>
+      </c>
+      <c r="E38">
+        <v>0.71</v>
+      </c>
+      <c r="F38">
+        <v>-0.8</v>
+      </c>
+      <c r="G38">
+        <f>$L$6*E38</f>
+        <v>31.633056</v>
+      </c>
+      <c r="H38">
+        <f>$L$6*F38</f>
+        <v>-35.642880000000005</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="12"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="13"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L38">
+        <f>G38+I38</f>
+        <v>39.652704</v>
+      </c>
+      <c r="M38">
+        <f>H38+J38</f>
+        <v>-43.662528000000009</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="15">
+      <c r="A40" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41">
+        <v>5</v>
+      </c>
+      <c r="B41" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41">
+        <f>F8*B6</f>
+        <v>60</v>
+      </c>
+      <c r="E41">
+        <v>0.83</v>
+      </c>
+      <c r="F41">
+        <v>-1.1299999999999999</v>
+      </c>
+      <c r="G41">
+        <f>$L$6*E41</f>
+        <v>36.979488000000003</v>
+      </c>
+      <c r="H41">
+        <f>$L$6*F41</f>
+        <v>-50.345568</v>
+      </c>
+      <c r="I41">
+        <f t="shared" ref="I41:I43" si="14">$L$6*$L$2</f>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J41">
+        <f t="shared" ref="J41:J43" si="15">-$L$6*$L$2</f>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L41">
+        <f>G41+I41</f>
+        <v>44.999136000000007</v>
+      </c>
+      <c r="M41">
+        <f>H41+J41</f>
+        <v>-58.365216000000004</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42">
+        <f>(B4-2*F8)*B6</f>
+        <v>480</v>
+      </c>
+      <c r="E42">
+        <v>0.7</v>
+      </c>
+      <c r="F42">
+        <v>-0.8</v>
+      </c>
+      <c r="G42">
+        <f>$L$6*E42</f>
+        <v>31.187519999999999</v>
+      </c>
+      <c r="H42">
+        <f>$L$6*F42</f>
+        <v>-35.642880000000005</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="14"/>
+        <v>8.0196480000000001</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="15"/>
+        <v>-8.0196480000000001</v>
+      </c>
+      <c r="L42">
+        <f>G42+I42</f>
+        <v>39.207167999999996</v>
+      </c>
+      <c r="M42">
+        <f>H42+J42</f>
+        <v>-43.662528000000009</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="B45">
+        <f>TAN($B$8*6.28/360)</f>
+        <v>0.2678069474078098</v>
+      </c>
+      <c r="C45">
+        <f>B45*F8</f>
+        <v>1.0712277896312392</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD8320E2-F01C-4F60-9B3D-82EC74076ADF}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25"/>

</xml_diff>